<commit_message>
remaining manually made changes of 0328
Signed-off-by: ibicdlcod <504161487@qq.com>
</commit_message>
<xml_diff>
--- a/doc/equip/Equip.xlsx
+++ b/doc/equip/Equip.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GuoMuoRuoProject\doc\equip\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AD1B06-5884-4BD3-9348-C724015D5E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81491F31-AC43-4384-9B9E-D16E7DC73612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Equip" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Equip!$A$2:$AF$585</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Equip!$A$2:$AG$585</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1789" uniqueCount="758">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1791" uniqueCount="760">
   <si>
     <t>id</t>
   </si>
@@ -2302,6 +2302,14 @@
   </si>
   <si>
     <t>JP-1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Storeprice</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>attr</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2552,7 +2560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF585"/>
+  <dimension ref="A1:AG585"/>
   <sheetFormatPr defaultColWidth="10.06640625" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.265625" customWidth="1"/>
@@ -2584,7 +2592,7 @@
     <col min="31" max="31" width="14.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2678,8 +2686,11 @@
       <c r="AF1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="AG1" s="1" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2776,8 +2787,11 @@
       <c r="AF2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="AG2" s="1" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2818,7 +2832,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2859,7 +2873,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2903,7 +2917,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2947,7 +2961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2988,7 +3002,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3029,7 +3043,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3070,7 +3084,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3111,7 +3125,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -3149,7 +3163,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -3193,7 +3207,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -3234,7 +3248,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -3275,7 +3289,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -3301,7 +3315,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -3878,7 +3892,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>31</v>
       </c>
@@ -3910,7 +3924,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>32</v>
       </c>
@@ -3942,7 +3956,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>33</v>
       </c>
@@ -3974,7 +3988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
@@ -4006,7 +4020,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>35</v>
       </c>
@@ -4038,7 +4052,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
@@ -4073,7 +4087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>37</v>
       </c>
@@ -4105,7 +4119,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>38</v>
       </c>
@@ -4134,7 +4148,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>39</v>
       </c>
@@ -4163,7 +4177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>40</v>
       </c>
@@ -4192,7 +4206,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>41</v>
       </c>
@@ -4221,7 +4235,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>42</v>
       </c>
@@ -4243,8 +4257,11 @@
       <c r="I44">
         <v>-1</v>
       </c>
-    </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AG44">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="45" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>43</v>
       </c>
@@ -4266,8 +4283,11 @@
       <c r="I45">
         <v>-1</v>
       </c>
-    </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AG45">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="46" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>44</v>
       </c>
@@ -4296,7 +4316,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45</v>
       </c>
@@ -4322,7 +4342,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>46</v>
       </c>
@@ -25478,7 +25498,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AF585" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:AG585" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
implement recon guided strike, sync fighter plane losses, various fixes
- Implement reconnaissance plane guided strike (触接): sort all fleet
  planes by Accuracy desc, trigger chance p=a*b/sqrt(1+b²) where a=air
  superiority, b=accuracy/100. First success amplifies all air attack
  damage by (1+accuracy/100)x. Applied to torpedo, dive, and cut-in.
- Fix fighter plane loss tracking: syncSquadronPlanes writes squadron
  plane counts (including fighters) back to slotPlanes after S1/S2/S3
  and air attacks, so replenishment cost covers all plane types
- Use u = max(0, u) instead of if(u<=0)u=0 for gunshot damage
- Show ship name before slot in battle report anti-air loss entries
- Set Firingspeed=1 for oxygen torpedoes (real-world reload devices)
  and all submarine torpedo tubes (inherent reload capacity)
</commit_message>
<xml_diff>
--- a/doc/equip/Equip.xlsx
+++ b/doc/equip/Equip.xlsx
@@ -2896,14 +2896,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AH585"/>
-  <sheetFormatPr defaultColWidth="5.27734375" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="5.1953125" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.81"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="5.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.81"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="32" min="6" style="1" width="5.28"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="33" style="2" width="5.28"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34.49"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="5.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.46"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="32" min="6" style="1" width="5.19"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="33" style="2" width="5.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3995,7 +3995,9 @@
       <c r="R17" s="6"/>
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
-      <c r="U17" s="6"/>
+      <c r="U17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V17" s="6"/>
       <c r="W17" s="5" t="n">
         <v>100</v>
@@ -6385,7 +6387,9 @@
       <c r="R60" s="6"/>
       <c r="S60" s="6"/>
       <c r="T60" s="6"/>
-      <c r="U60" s="6"/>
+      <c r="U60" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V60" s="6"/>
       <c r="W60" s="5" t="n">
         <v>120</v>
@@ -8521,7 +8525,9 @@
       <c r="R96" s="6"/>
       <c r="S96" s="6"/>
       <c r="T96" s="6"/>
-      <c r="U96" s="6"/>
+      <c r="U96" s="5" t="n">
+        <v>12</v>
+      </c>
       <c r="V96" s="6"/>
       <c r="W96" s="5" t="n">
         <v>160</v>
@@ -10333,7 +10339,9 @@
       <c r="R126" s="6"/>
       <c r="S126" s="6"/>
       <c r="T126" s="6"/>
-      <c r="U126" s="6"/>
+      <c r="U126" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V126" s="6"/>
       <c r="W126" s="5" t="n">
         <v>80</v>
@@ -10445,7 +10453,9 @@
       <c r="R128" s="6"/>
       <c r="S128" s="6"/>
       <c r="T128" s="6"/>
-      <c r="U128" s="6"/>
+      <c r="U128" s="6" t="n">
+        <v>16</v>
+      </c>
       <c r="V128" s="6"/>
       <c r="W128" s="5" t="n">
         <v>124</v>
@@ -13515,7 +13525,9 @@
       <c r="R180" s="6"/>
       <c r="S180" s="6"/>
       <c r="T180" s="6"/>
-      <c r="U180" s="6"/>
+      <c r="U180" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V180" s="6"/>
       <c r="W180" s="5" t="n">
         <v>135</v>
@@ -15575,7 +15587,9 @@
       <c r="R214" s="6"/>
       <c r="S214" s="6"/>
       <c r="T214" s="6"/>
-      <c r="U214" s="6"/>
+      <c r="U214" s="6" t="n">
+        <v>16</v>
+      </c>
       <c r="V214" s="6"/>
       <c r="W214" s="5" t="n">
         <v>150</v>
@@ -15631,7 +15645,9 @@
       </c>
       <c r="S215" s="6"/>
       <c r="T215" s="6"/>
-      <c r="U215" s="6"/>
+      <c r="U215" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="V215" s="6"/>
       <c r="W215" s="5" t="n">
         <v>153</v>
@@ -19942,7 +19958,9 @@
       <c r="R286" s="6"/>
       <c r="S286" s="6"/>
       <c r="T286" s="6"/>
-      <c r="U286" s="6"/>
+      <c r="U286" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V286" s="6"/>
       <c r="W286" s="5" t="n">
         <v>90</v>
@@ -19998,7 +20016,9 @@
       <c r="R287" s="6"/>
       <c r="S287" s="6"/>
       <c r="T287" s="6"/>
-      <c r="U287" s="6"/>
+      <c r="U287" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V287" s="6"/>
       <c r="W287" s="5" t="n">
         <v>110</v>
@@ -25796,7 +25816,9 @@
       <c r="R381" s="6"/>
       <c r="S381" s="6"/>
       <c r="T381" s="6"/>
-      <c r="U381" s="6"/>
+      <c r="U381" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="V381" s="6"/>
       <c r="W381" s="5" t="n">
         <v>192</v>
@@ -29336,7 +29358,9 @@
       <c r="R438" s="6"/>
       <c r="S438" s="6"/>
       <c r="T438" s="6"/>
-      <c r="U438" s="6"/>
+      <c r="U438" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="V438" s="6"/>
       <c r="W438" s="5" t="n">
         <v>100</v>
@@ -29390,7 +29414,9 @@
       <c r="R439" s="6"/>
       <c r="S439" s="6"/>
       <c r="T439" s="6"/>
-      <c r="U439" s="6"/>
+      <c r="U439" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="V439" s="6"/>
       <c r="W439" s="5" t="n">
         <v>140</v>
@@ -29446,7 +29472,9 @@
       <c r="R440" s="6"/>
       <c r="S440" s="6"/>
       <c r="T440" s="6"/>
-      <c r="U440" s="6"/>
+      <c r="U440" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="V440" s="6"/>
       <c r="W440" s="5" t="n">
         <v>62</v>
@@ -29500,7 +29528,9 @@
       <c r="R441" s="6"/>
       <c r="S441" s="6"/>
       <c r="T441" s="6"/>
-      <c r="U441" s="6"/>
+      <c r="U441" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="V441" s="6"/>
       <c r="W441" s="5" t="n">
         <v>94</v>
@@ -30292,7 +30322,9 @@
       <c r="R454" s="6"/>
       <c r="S454" s="6"/>
       <c r="T454" s="6"/>
-      <c r="U454" s="6"/>
+      <c r="U454" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="V454" s="6"/>
       <c r="W454" s="5" t="n">
         <v>120</v>
@@ -30536,7 +30568,9 @@
       </c>
       <c r="S458" s="6"/>
       <c r="T458" s="6"/>
-      <c r="U458" s="6"/>
+      <c r="U458" s="6" t="n">
+        <v>24</v>
+      </c>
       <c r="V458" s="6"/>
       <c r="W458" s="5" t="n">
         <v>135</v>
@@ -33540,7 +33574,9 @@
       <c r="R507" s="6"/>
       <c r="S507" s="6"/>
       <c r="T507" s="6"/>
-      <c r="U507" s="6"/>
+      <c r="U507" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="V507" s="6"/>
       <c r="W507" s="5" t="n">
         <v>78</v>
@@ -33594,7 +33630,9 @@
       <c r="R508" s="6"/>
       <c r="S508" s="6"/>
       <c r="T508" s="6"/>
-      <c r="U508" s="6"/>
+      <c r="U508" s="6" t="n">
+        <v>20</v>
+      </c>
       <c r="V508" s="6"/>
       <c r="W508" s="5" t="n">
         <v>124</v>

</xml_diff>